<commit_message>
Loading the same packages across all scripts for consistency, and adding code to plot all synergy/viability plots together as a single figure
</commit_message>
<xml_diff>
--- a/4_output/Loewe_synergy_response_data.xlsx
+++ b/4_output/Loewe_synergy_response_data.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Adavosertib" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Zorifertinib" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="AZD7762" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="BI-2536" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="BI2536" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Entinostat" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Gefitinib" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Sapitinib" sheetId="7" state="visible" r:id="rId7"/>
@@ -71,13 +71,13 @@
     <t xml:space="preserve">AZD7762_sem</t>
   </si>
   <si>
-    <t xml:space="preserve">BI-2536_conc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BI-2536_response</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BI-2536_sem</t>
+    <t xml:space="preserve">BI2536_conc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BI2536_response</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BI2536_sem</t>
   </si>
   <si>
     <t xml:space="preserve">Entinostat_conc</t>

</xml_diff>